<commit_message>
feat: audit A1/A2 vocabulary with Oxford 3000/5000 CEFR standards, improve progress bar contrast, and enforce strict deploy rule
</commit_message>
<xml_diff>
--- a/docs/A1-1000.xlsx
+++ b/docs/A1-1000.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -513,13 +513,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Click</v>
+        <v>Post</v>
       </c>
       <c r="B9" t="str">
-        <v>Tıklamak</v>
+        <v>Gönderi, Paylaşım</v>
       </c>
       <c r="C9" t="str">
-        <v>Verb / Noun</v>
+        <v>Noun</v>
       </c>
       <c r="D9" t="str">
         <v>Communication and Technology</v>
@@ -653,10 +653,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Keyboard</v>
+        <v>News</v>
       </c>
       <c r="B19" t="str">
-        <v>Klavye</v>
+        <v>Haberler</v>
       </c>
       <c r="C19" t="str">
         <v>Noun</v>
@@ -709,10 +709,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Password</v>
+        <v>Dialogue</v>
       </c>
       <c r="B23" t="str">
-        <v>Şifre, Parola</v>
+        <v>Diyalog</v>
       </c>
       <c r="C23" t="str">
         <v>Noun</v>
@@ -765,10 +765,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Software</v>
+        <v>Sound</v>
       </c>
       <c r="B27" t="str">
-        <v>Yazılım</v>
+        <v>Ses</v>
       </c>
       <c r="C27" t="str">
         <v>Noun</v>
@@ -1073,10 +1073,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Notebook</v>
+        <v>Page</v>
       </c>
       <c r="B49" t="str">
-        <v>Not defteri</v>
+        <v>Sayfa</v>
       </c>
       <c r="C49" t="str">
         <v>Noun</v>
@@ -1157,10 +1157,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Receipt</v>
+        <v>List</v>
       </c>
       <c r="B55" t="str">
-        <v>Fiş, Makbuz</v>
+        <v>Liste</v>
       </c>
       <c r="C55" t="str">
         <v>Noun</v>
@@ -1185,10 +1185,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Textbook</v>
+        <v>Title</v>
       </c>
       <c r="B57" t="str">
-        <v>Ders kitabı</v>
+        <v>Başlık</v>
       </c>
       <c r="C57" t="str">
         <v>Noun</v>
@@ -1241,10 +1241,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Biology</v>
+        <v>Art</v>
       </c>
       <c r="B61" t="str">
-        <v>Biyoloji</v>
+        <v>Sanat, Resim dersi</v>
       </c>
       <c r="C61" t="str">
         <v>Noun</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Chemistry</v>
+        <v>Reading</v>
       </c>
       <c r="B65" t="str">
-        <v>Kimya</v>
+        <v>Okuma</v>
       </c>
       <c r="C65" t="str">
         <v>Noun</v>
@@ -1437,10 +1437,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Examination</v>
+        <v>Project</v>
       </c>
       <c r="B75" t="str">
-        <v>Muayene, Sınav</v>
+        <v>Proje</v>
       </c>
       <c r="C75" t="str">
         <v>Noun</v>
@@ -1521,10 +1521,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Instruction</v>
+        <v>Rule</v>
       </c>
       <c r="B81" t="str">
-        <v>Talimat, Yönerge</v>
+        <v>Kural</v>
       </c>
       <c r="C81" t="str">
         <v>Noun</v>
@@ -1549,10 +1549,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Knowledge</v>
+        <v>Meaning</v>
       </c>
       <c r="B83" t="str">
-        <v>Bilgi</v>
+        <v>Anlam</v>
       </c>
       <c r="C83" t="str">
         <v>Noun</v>
@@ -1619,10 +1619,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Level</v>
+        <v>Topic</v>
       </c>
       <c r="B88" t="str">
-        <v>Seviye</v>
+        <v>Konu</v>
       </c>
       <c r="C88" t="str">
         <v>Noun</v>
@@ -1717,10 +1717,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Physics</v>
+        <v>Writing</v>
       </c>
       <c r="B95" t="str">
-        <v>Fizik</v>
+        <v>Yazma</v>
       </c>
       <c r="C95" t="str">
         <v>Noun</v>
@@ -1955,13 +1955,13 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Bake</v>
+        <v>Cooking</v>
       </c>
       <c r="B112" t="str">
-        <v>Fırında pişirmek</v>
+        <v>Yemek pişirme</v>
       </c>
       <c r="C112" t="str">
-        <v>Verb</v>
+        <v>Noun</v>
       </c>
       <c r="D112" t="str">
         <v>Food and Drink</v>
@@ -3845,10 +3845,10 @@
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Lip</v>
+        <v>Feeling</v>
       </c>
       <c r="B247" t="str">
-        <v>Dudak</v>
+        <v>His, Duygu</v>
       </c>
       <c r="C247" t="str">
         <v>Noun</v>
@@ -4041,10 +4041,10 @@
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>Tissue</v>
+        <v>Life</v>
       </c>
       <c r="B261" t="str">
-        <v>Peçete, Doku</v>
+        <v>Yaşam, Hayat</v>
       </c>
       <c r="C261" t="str">
         <v>Noun</v>
@@ -4055,13 +4055,13 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>Toe</v>
+        <v>Relax</v>
       </c>
       <c r="B262" t="str">
-        <v>Ayak parmağı</v>
+        <v>Rahatlamak, Dinlenmek</v>
       </c>
       <c r="C262" t="str">
-        <v>Noun</v>
+        <v>Verb</v>
       </c>
       <c r="D262" t="str">
         <v>Health and Body</v>
@@ -4069,13 +4069,13 @@
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>Tongue</v>
+        <v>Born</v>
       </c>
       <c r="B263" t="str">
-        <v>Dil (Organ)</v>
+        <v>Doğmuş, Dünyaya gelmiş</v>
       </c>
       <c r="C263" t="str">
-        <v>Noun</v>
+        <v>Adjective</v>
       </c>
       <c r="D263" t="str">
         <v>Health and Body</v>
@@ -4251,10 +4251,10 @@
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>Blanket</v>
+        <v>Wall</v>
       </c>
       <c r="B276" t="str">
-        <v>Battaniye</v>
+        <v>Duvar</v>
       </c>
       <c r="C276" t="str">
         <v>Noun</v>
@@ -4279,10 +4279,10 @@
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>Cabinet</v>
+        <v>Box</v>
       </c>
       <c r="B278" t="str">
-        <v>Dolap</v>
+        <v>Kutu</v>
       </c>
       <c r="C278" t="str">
         <v>Noun</v>
@@ -4307,10 +4307,10 @@
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>Ceiling</v>
+        <v>Home</v>
       </c>
       <c r="B280" t="str">
-        <v>Tavan</v>
+        <v>Ev, Yuva</v>
       </c>
       <c r="C280" t="str">
         <v>Noun</v>
@@ -4391,10 +4391,10 @@
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>Entrance</v>
+        <v>Front</v>
       </c>
       <c r="B286" t="str">
-        <v>Giriş</v>
+        <v>Ön taraf, Ön cephe</v>
       </c>
       <c r="C286" t="str">
         <v>Noun</v>
@@ -4461,13 +4461,13 @@
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>Garage</v>
+        <v>Downstairs</v>
       </c>
       <c r="B291" t="str">
-        <v>Garaj</v>
+        <v>Alt kat</v>
       </c>
       <c r="C291" t="str">
-        <v>Noun</v>
+        <v>Adverb</v>
       </c>
       <c r="D291" t="str">
         <v>House and Home</v>
@@ -4517,10 +4517,10 @@
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>Heating</v>
+        <v>Space</v>
       </c>
       <c r="B295" t="str">
-        <v>Isıtma sistemi</v>
+        <v>Alan, Yer</v>
       </c>
       <c r="C295" t="str">
         <v>Noun</v>
@@ -4727,10 +4727,10 @@
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>Shelf</v>
+        <v>Place</v>
       </c>
       <c r="B310" t="str">
-        <v>Raf</v>
+        <v>Yer, Mekan</v>
       </c>
       <c r="C310" t="str">
         <v>Noun</v>
@@ -4755,10 +4755,10 @@
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>Sink</v>
+        <v>Outside</v>
       </c>
       <c r="B312" t="str">
-        <v>Evye</v>
+        <v>Dışarısı, Bahçe</v>
       </c>
       <c r="C312" t="str">
         <v>Noun</v>
@@ -5035,10 +5035,10 @@
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>Drum</v>
+        <v>Game</v>
       </c>
       <c r="B332" t="str">
-        <v>Davul</v>
+        <v>Oyun</v>
       </c>
       <c r="C332" t="str">
         <v>Noun</v>
@@ -5413,10 +5413,10 @@
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>Studio</v>
+        <v>Theatre</v>
       </c>
       <c r="B359" t="str">
-        <v>Stüdyo</v>
+        <v>Tiyatro</v>
       </c>
       <c r="C359" t="str">
         <v>Noun</v>
@@ -5469,10 +5469,10 @@
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>Tune</v>
+        <v>Fun</v>
       </c>
       <c r="B363" t="str">
-        <v>Melodi</v>
+        <v>Eğlence</v>
       </c>
       <c r="C363" t="str">
         <v>Noun</v>
@@ -5609,10 +5609,10 @@
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>Bee</v>
+        <v>Flower</v>
       </c>
       <c r="B373" t="str">
-        <v>Arı</v>
+        <v>Çiçek</v>
       </c>
       <c r="C373" t="str">
         <v>Noun</v>
@@ -5945,10 +5945,10 @@
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>Leaf</v>
+        <v>World</v>
       </c>
       <c r="B397" t="str">
-        <v>Yaprak</v>
+        <v>Dünya</v>
       </c>
       <c r="C397" t="str">
         <v>Noun</v>
@@ -5987,10 +5987,10 @@
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>Monster</v>
+        <v>Fire</v>
       </c>
       <c r="B400" t="str">
-        <v>Canavar</v>
+        <v>Ateş</v>
       </c>
       <c r="C400" t="str">
         <v>Noun</v>
@@ -6057,10 +6057,10 @@
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>Nest</v>
+        <v>Farm</v>
       </c>
       <c r="B405" t="str">
-        <v>Yuva</v>
+        <v>Çiftlik</v>
       </c>
       <c r="C405" t="str">
         <v>Noun</v>
@@ -6883,10 +6883,10 @@
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>Friendship</v>
+        <v>Group</v>
       </c>
       <c r="B464" t="str">
-        <v>Dostluk</v>
+        <v>Grup, Topluluk</v>
       </c>
       <c r="C464" t="str">
         <v>Noun</v>
@@ -7401,10 +7401,10 @@
     </row>
     <row r="501">
       <c r="A501" t="str">
-        <v>Stranger</v>
+        <v>Neighbour</v>
       </c>
       <c r="B501" t="str">
-        <v>Yabancı</v>
+        <v>Komşu</v>
       </c>
       <c r="C501" t="str">
         <v>Noun</v>
@@ -7569,10 +7569,10 @@
     </row>
     <row r="513">
       <c r="A513" t="str">
-        <v>Youth</v>
+        <v>Team</v>
       </c>
       <c r="B513" t="str">
-        <v>Gençlik</v>
+        <v>Takım, Ekip</v>
       </c>
       <c r="C513" t="str">
         <v>Noun</v>
@@ -7639,10 +7639,10 @@
     </row>
     <row r="518">
       <c r="A518" t="str">
-        <v>Cap</v>
+        <v>Bag</v>
       </c>
       <c r="B518" t="str">
-        <v>Şapka, Kep</v>
+        <v>Çanta, Poşet</v>
       </c>
       <c r="C518" t="str">
         <v>Noun</v>
@@ -7751,10 +7751,10 @@
     </row>
     <row r="526">
       <c r="A526" t="str">
-        <v>Coin</v>
+        <v>Money</v>
       </c>
       <c r="B526" t="str">
-        <v>Bozuk para</v>
+        <v>Para</v>
       </c>
       <c r="C526" t="str">
         <v>Noun</v>
@@ -7779,10 +7779,10 @@
     </row>
     <row r="528">
       <c r="A528" t="str">
-        <v>Cotton</v>
+        <v>Product</v>
       </c>
       <c r="B528" t="str">
-        <v>Pamuk</v>
+        <v>Ürün</v>
       </c>
       <c r="C528" t="str">
         <v>Noun</v>
@@ -7807,10 +7807,10 @@
     </row>
     <row r="530">
       <c r="A530" t="str">
-        <v>Costume</v>
+        <v>Pair</v>
       </c>
       <c r="B530" t="str">
-        <v>Kostüm</v>
+        <v>Çift</v>
       </c>
       <c r="C530" t="str">
         <v>Noun</v>
@@ -7821,10 +7821,10 @@
     </row>
     <row r="531">
       <c r="A531" t="str">
-        <v>Discount</v>
+        <v>Order</v>
       </c>
       <c r="B531" t="str">
-        <v>İndirim</v>
+        <v>Sipariş</v>
       </c>
       <c r="C531" t="str">
         <v>Noun</v>
@@ -7891,10 +7891,10 @@
     </row>
     <row r="536">
       <c r="A536" t="str">
-        <v>Glove</v>
+        <v>Piece</v>
       </c>
       <c r="B536" t="str">
-        <v>Eldiven</v>
+        <v>Parça, Tane</v>
       </c>
       <c r="C536" t="str">
         <v>Noun</v>
@@ -7975,10 +7975,10 @@
     </row>
     <row r="542">
       <c r="A542" t="str">
-        <v>Leather</v>
+        <v>Style</v>
       </c>
       <c r="B542" t="str">
-        <v>Deri</v>
+        <v>Tarz, Stil</v>
       </c>
       <c r="C542" t="str">
         <v>Noun</v>
@@ -8031,10 +8031,10 @@
     </row>
     <row r="546">
       <c r="A546" t="str">
-        <v>Package</v>
+        <v>Bank</v>
       </c>
       <c r="B546" t="str">
-        <v>Paket</v>
+        <v>Banka</v>
       </c>
       <c r="C546" t="str">
         <v>Noun</v>
@@ -8143,13 +8143,13 @@
     </row>
     <row r="554">
       <c r="A554" t="str">
-        <v>Rent</v>
+        <v>Choose</v>
       </c>
       <c r="B554" t="str">
-        <v>Kiralamak</v>
+        <v>Seçmek</v>
       </c>
       <c r="C554" t="str">
-        <v>Verb / Noun</v>
+        <v>Verb</v>
       </c>
       <c r="D554" t="str">
         <v>Shopping and Clothes</v>
@@ -8465,10 +8465,10 @@
     </row>
     <row r="577">
       <c r="A577" t="str">
-        <v>Wool</v>
+        <v>Colour</v>
       </c>
       <c r="B577" t="str">
-        <v>Yün</v>
+        <v>Renk</v>
       </c>
       <c r="C577" t="str">
         <v>Noun</v>
@@ -8633,13 +8633,13 @@
     </row>
     <row r="589">
       <c r="A589" t="str">
-        <v>Kick</v>
+        <v>Ball</v>
       </c>
       <c r="B589" t="str">
-        <v>Tekmelemek</v>
+        <v>Top</v>
       </c>
       <c r="C589" t="str">
-        <v>Verb / Noun</v>
+        <v>Noun</v>
       </c>
       <c r="D589" t="str">
         <v>Sports and Hobbies</v>
@@ -9333,10 +9333,10 @@
     </row>
     <row r="639">
       <c r="A639" t="str">
-        <v>Helicopter</v>
+        <v>City</v>
       </c>
       <c r="B639" t="str">
-        <v>Helikopter</v>
+        <v>Şehir, Kent</v>
       </c>
       <c r="C639" t="str">
         <v>Noun</v>
@@ -9487,10 +9487,10 @@
     </row>
     <row r="650">
       <c r="A650" t="str">
-        <v>Path</v>
+        <v>Country</v>
       </c>
       <c r="B650" t="str">
-        <v>Yol, Patika</v>
+        <v>Ülke</v>
       </c>
       <c r="C650" t="str">
         <v>Noun</v>
@@ -9767,10 +9767,10 @@
     </row>
     <row r="670">
       <c r="A670" t="str">
-        <v>Tunnel</v>
+        <v>Town</v>
       </c>
       <c r="B670" t="str">
-        <v>Tünel</v>
+        <v>Kasaba</v>
       </c>
       <c r="C670" t="str">
         <v>Noun</v>
@@ -10215,10 +10215,10 @@
     </row>
     <row r="702">
       <c r="A702" t="str">
-        <v>Mechanic</v>
+        <v>Meeting</v>
       </c>
       <c r="B702" t="str">
-        <v>Tamirci</v>
+        <v>Toplantı</v>
       </c>
       <c r="C702" t="str">
         <v>Noun</v>
@@ -10243,10 +10243,10 @@
     </row>
     <row r="704">
       <c r="A704" t="str">
-        <v>Occupation</v>
+        <v>Plan</v>
       </c>
       <c r="B704" t="str">
-        <v>Meslek</v>
+        <v>Plan</v>
       </c>
       <c r="C704" t="str">
         <v>Noun</v>
@@ -10299,10 +10299,10 @@
     </row>
     <row r="708">
       <c r="A708" t="str">
-        <v>Photographer</v>
+        <v>Report</v>
       </c>
       <c r="B708" t="str">
-        <v>Fotoğrafçı</v>
+        <v>Rapor</v>
       </c>
       <c r="C708" t="str">
         <v>Noun</v>
@@ -10397,10 +10397,10 @@
     </row>
     <row r="715">
       <c r="A715" t="str">
-        <v>Staff</v>
+        <v>Programme</v>
       </c>
       <c r="B715" t="str">
-        <v>Personel</v>
+        <v>Program</v>
       </c>
       <c r="C715" t="str">
         <v>Noun</v>
@@ -10873,10 +10873,10 @@
     </row>
     <row r="749">
       <c r="A749" t="str">
-        <v>Noon</v>
+        <v>Date</v>
       </c>
       <c r="B749" t="str">
-        <v>Öğle vakti</v>
+        <v>Tarih</v>
       </c>
       <c r="C749" t="str">
         <v>Noun</v>
@@ -11041,13 +11041,13 @@
     </row>
     <row r="761">
       <c r="A761" t="str">
-        <v>Weekly</v>
+        <v>Period</v>
       </c>
       <c r="B761" t="str">
-        <v>Haftalık</v>
+        <v>Dönem, Süre</v>
       </c>
       <c r="C761" t="str">
-        <v>Adjective / Adverb</v>
+        <v>Noun</v>
       </c>
       <c r="D761" t="str">
         <v>Time and Dates</v>
@@ -11055,13 +11055,13 @@
     </row>
     <row r="762">
       <c r="A762" t="str">
-        <v>Monthly</v>
+        <v>Moment</v>
       </c>
       <c r="B762" t="str">
-        <v>Aylık</v>
+        <v>An, Kısa süre</v>
       </c>
       <c r="C762" t="str">
-        <v>Adjective / Adverb</v>
+        <v>Noun</v>
       </c>
       <c r="D762" t="str">
         <v>Time and Dates</v>
@@ -12357,13 +12357,13 @@
     </row>
     <row r="855">
       <c r="A855" t="str">
-        <v>Total</v>
+        <v>Number</v>
       </c>
       <c r="B855" t="str">
-        <v>Toplam</v>
+        <v>Sayı, Numara</v>
       </c>
       <c r="C855" t="str">
-        <v>Adjective / Noun</v>
+        <v>Noun</v>
       </c>
       <c r="D855" t="str">
         <v>Numbers and Quantities</v>
@@ -12427,10 +12427,10 @@
     </row>
     <row r="860">
       <c r="A860" t="str">
-        <v>Tiny</v>
+        <v>Difficult</v>
       </c>
       <c r="B860" t="str">
-        <v>Minik</v>
+        <v>Zor, Güç</v>
       </c>
       <c r="C860" t="str">
         <v>Adjective</v>
@@ -12497,10 +12497,10 @@
     </row>
     <row r="865">
       <c r="A865" t="str">
-        <v>Broad</v>
+        <v>Famous</v>
       </c>
       <c r="B865" t="str">
-        <v>Geniş</v>
+        <v>Ünlü, Meşhur</v>
       </c>
       <c r="C865" t="str">
         <v>Adjective</v>
@@ -12707,10 +12707,10 @@
     </row>
     <row r="880">
       <c r="A880" t="str">
-        <v>Complex</v>
+        <v>Busy</v>
       </c>
       <c r="B880" t="str">
-        <v>Karmaşık</v>
+        <v>Meşgul, Yoğun</v>
       </c>
       <c r="C880" t="str">
         <v>Adjective</v>
@@ -12987,10 +12987,10 @@
     </row>
     <row r="900">
       <c r="A900" t="str">
-        <v>Cute</v>
+        <v>Cool</v>
       </c>
       <c r="B900" t="str">
-        <v>Tatlı, Sevimli</v>
+        <v>Harika, Havalı</v>
       </c>
       <c r="C900" t="str">
         <v>Adjective</v>
@@ -13001,10 +13001,10 @@
     </row>
     <row r="901">
       <c r="A901" t="str">
-        <v>Ugly</v>
+        <v>Afraid</v>
       </c>
       <c r="B901" t="str">
-        <v>Çirkin</v>
+        <v>Korkmuş</v>
       </c>
       <c r="C901" t="str">
         <v>Adjective</v>
@@ -13353,8 +13353,8 @@
       <c r="A926" t="str">
         <v>True</v>
       </c>
-      <c r="B926" t="b">
-        <v>1</v>
+      <c r="B926" t="str">
+        <v>Doğru</v>
       </c>
       <c r="C926" t="str">
         <v>Adjective</v>
@@ -13367,8 +13367,8 @@
       <c r="A927" t="str">
         <v>Wrong</v>
       </c>
-      <c r="B927" t="b">
-        <v>0</v>
+      <c r="B927" t="str">
+        <v>Yanlış</v>
       </c>
       <c r="C927" t="str">
         <v>Adjective</v>
@@ -13463,10 +13463,10 @@
     </row>
     <row r="934">
       <c r="A934" t="str">
-        <v>Rough</v>
+        <v>Ready</v>
       </c>
       <c r="B934" t="str">
-        <v>Pürüzlü, Kaba</v>
+        <v>Hazır</v>
       </c>
       <c r="C934" t="str">
         <v>Adjective</v>

</xml_diff>